<commit_message>
chore: run 2026-04-08 10:19 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_08_04_2026.xlsx
+++ b/logs/Consolidado_08_04_2026.xlsx
@@ -641,7 +641,7 @@
         <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -676,10 +676,10 @@
         <v>77</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -736,7 +736,7 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
@@ -11529,40 +11529,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>08/04/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Cupuaçu Reparing Very Dry Hair Shampoo
 Champô Cupuaçu BIO Repara Cabelo Muito Seco
 400 ml</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-reparing-very-dry-hair-shampoo-343983.html</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>7104602</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>

</xml_diff>